<commit_message>
Updated BECF, EIaE, BIFUbCCS, ARpUIiRC, BCRbQ, and CRbQ
</commit_message>
<xml_diff>
--- a/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
+++ b/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BCRbQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D60CC50-7280-3E47-BB25-89FDB285D75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B75B75E-3EC5-C94B-8289-46E0840638AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="coal retirement" sheetId="2" r:id="rId2"/>
-    <sheet name="BCRbQ" sheetId="3" r:id="rId3"/>
+    <sheet name="Computation" sheetId="4" r:id="rId3"/>
+    <sheet name="BCRbQ" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>BCRbQ BAU Capacity Retirements before Quantization</t>
   </si>
@@ -3229,6 +3230,424 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBE85BC8-7BD0-D94C-AAB8-BCEB0307B5FB}">
+  <dimension ref="A1:BA8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="7">
+        <v>2019</v>
+      </c>
+      <c r="C1" s="7">
+        <v>2020</v>
+      </c>
+      <c r="D1" s="7">
+        <v>2021</v>
+      </c>
+      <c r="E1" s="7">
+        <v>2022</v>
+      </c>
+      <c r="F1" s="7">
+        <v>2023</v>
+      </c>
+      <c r="G1" s="7">
+        <v>2024</v>
+      </c>
+      <c r="H1" s="7">
+        <v>2025</v>
+      </c>
+      <c r="I1" s="7">
+        <v>2026</v>
+      </c>
+      <c r="J1" s="7">
+        <v>2027</v>
+      </c>
+      <c r="K1" s="7">
+        <v>2028</v>
+      </c>
+      <c r="L1" s="7">
+        <v>2029</v>
+      </c>
+      <c r="M1" s="7">
+        <v>2030</v>
+      </c>
+      <c r="N1" s="7">
+        <v>2031</v>
+      </c>
+      <c r="O1" s="7">
+        <v>2032</v>
+      </c>
+      <c r="P1" s="7">
+        <v>2033</v>
+      </c>
+      <c r="Q1" s="7">
+        <v>2034</v>
+      </c>
+      <c r="R1" s="7">
+        <v>2035</v>
+      </c>
+      <c r="S1" s="7">
+        <v>2036</v>
+      </c>
+      <c r="T1" s="7">
+        <v>2037</v>
+      </c>
+      <c r="U1" s="7">
+        <v>2038</v>
+      </c>
+      <c r="V1" s="7">
+        <v>2039</v>
+      </c>
+      <c r="W1" s="7">
+        <v>2040</v>
+      </c>
+      <c r="X1" s="7">
+        <v>2041</v>
+      </c>
+      <c r="Y1" s="7">
+        <v>2042</v>
+      </c>
+      <c r="Z1" s="7">
+        <v>2043</v>
+      </c>
+      <c r="AA1" s="7">
+        <v>2044</v>
+      </c>
+      <c r="AB1" s="7">
+        <v>2045</v>
+      </c>
+      <c r="AC1" s="7">
+        <v>2046</v>
+      </c>
+      <c r="AD1" s="7">
+        <v>2047</v>
+      </c>
+      <c r="AE1" s="7">
+        <v>2048</v>
+      </c>
+      <c r="AF1" s="7">
+        <v>2049</v>
+      </c>
+      <c r="AG1" s="7">
+        <v>2050</v>
+      </c>
+      <c r="AH1" s="7">
+        <v>2051</v>
+      </c>
+      <c r="AI1" s="7">
+        <v>2052</v>
+      </c>
+      <c r="AJ1" s="7">
+        <v>2053</v>
+      </c>
+      <c r="AK1" s="7">
+        <v>2054</v>
+      </c>
+      <c r="AL1" s="7">
+        <v>2055</v>
+      </c>
+      <c r="AM1" s="7">
+        <v>2056</v>
+      </c>
+      <c r="AN1" s="7">
+        <v>2057</v>
+      </c>
+      <c r="AO1" s="7">
+        <v>2058</v>
+      </c>
+      <c r="AP1" s="7">
+        <v>2059</v>
+      </c>
+      <c r="AQ1" s="7">
+        <v>2060</v>
+      </c>
+      <c r="AR1" s="7">
+        <v>2061</v>
+      </c>
+      <c r="AS1" s="7">
+        <v>2062</v>
+      </c>
+      <c r="AT1" s="7">
+        <v>2063</v>
+      </c>
+      <c r="AU1" s="7">
+        <v>2064</v>
+      </c>
+      <c r="AV1" s="7">
+        <v>2065</v>
+      </c>
+      <c r="AW1" s="7">
+        <v>2066</v>
+      </c>
+      <c r="AX1" s="7">
+        <v>2067</v>
+      </c>
+      <c r="AY1" s="7">
+        <v>2068</v>
+      </c>
+      <c r="AZ1" s="7">
+        <v>2069</v>
+      </c>
+      <c r="BA1" s="7">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="10">
+        <f>C7/7</f>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="C2" s="10">
+        <f>B2</f>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="D2" s="10">
+        <f t="shared" ref="D2:H2" si="0">C2</f>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="E2" s="10">
+        <f t="shared" si="0"/>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="F2" s="10">
+        <f t="shared" si="0"/>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="G2" s="10">
+        <f t="shared" si="0"/>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="H2" s="10">
+        <f t="shared" si="0"/>
+        <v>157.14285714285714</v>
+      </c>
+      <c r="I2" s="10">
+        <f>D7/5</f>
+        <v>200</v>
+      </c>
+      <c r="J2" s="10">
+        <f t="shared" ref="J2:L2" si="1">I2</f>
+        <v>200</v>
+      </c>
+      <c r="K2" s="10">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="L2" s="10">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="M2" s="10">
+        <f>L2</f>
+        <v>200</v>
+      </c>
+      <c r="N2" s="10">
+        <f>E7/5</f>
+        <v>1800</v>
+      </c>
+      <c r="O2" s="10">
+        <f>N2</f>
+        <v>1800</v>
+      </c>
+      <c r="P2" s="10">
+        <f t="shared" ref="P2:R2" si="2">O2</f>
+        <v>1800</v>
+      </c>
+      <c r="Q2" s="10">
+        <f t="shared" si="2"/>
+        <v>1800</v>
+      </c>
+      <c r="R2" s="10">
+        <f t="shared" si="2"/>
+        <v>1800</v>
+      </c>
+      <c r="S2" s="10">
+        <f>F7/5</f>
+        <v>4800</v>
+      </c>
+      <c r="T2" s="10">
+        <f>S2</f>
+        <v>4800</v>
+      </c>
+      <c r="U2" s="10">
+        <f t="shared" ref="U2:W2" si="3">T2</f>
+        <v>4800</v>
+      </c>
+      <c r="V2" s="10">
+        <f t="shared" si="3"/>
+        <v>4800</v>
+      </c>
+      <c r="W2" s="10">
+        <f t="shared" si="3"/>
+        <v>4800</v>
+      </c>
+      <c r="X2" s="10">
+        <f>G7/15</f>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="Y2" s="10">
+        <f>X2</f>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="Z2" s="10">
+        <f t="shared" ref="Z2:AL2" si="4">Y2</f>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AA2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AB2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AC2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AD2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AE2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AF2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AG2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AH2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AI2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AJ2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AK2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AL2" s="10">
+        <f t="shared" si="4"/>
+        <v>333.33333333333331</v>
+      </c>
+      <c r="AM2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AS2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AT2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AU2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AV2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AX2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AY2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AZ2" s="10">
+        <v>0</v>
+      </c>
+      <c r="BA2" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2030</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2035</v>
+      </c>
+      <c r="F6" s="5">
+        <v>2040</v>
+      </c>
+      <c r="G6" s="5">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="7" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7">
+        <v>1100</v>
+      </c>
+      <c r="D7">
+        <v>1000</v>
+      </c>
+      <c r="E7">
+        <v>9000</v>
+      </c>
+      <c r="F7">
+        <v>24000</v>
+      </c>
+      <c r="G7">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="I2 N2 S2 X2" formula="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF1E4E79"/>
@@ -3407,42 +3826,52 @@
         <v>15</v>
       </c>
       <c r="B2" s="10">
-        <v>0</v>
+        <f>Computation!B2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="C2" s="10">
-        <v>0</v>
+        <f>Computation!C2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="D2" s="10">
-        <v>0</v>
+        <f>Computation!D2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="E2" s="10">
-        <v>0</v>
+        <f>Computation!E2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="F2" s="10">
-        <v>0</v>
+        <f>Computation!F2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="G2" s="10">
-        <v>0</v>
+        <f>Computation!G2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="H2" s="10">
-        <f>'coal retirement'!C42</f>
-        <v>4200</v>
+        <f>Computation!H2</f>
+        <v>157.14285714285714</v>
       </c>
       <c r="I2" s="10">
-        <v>0</v>
+        <f>Computation!I2</f>
+        <v>200</v>
       </c>
       <c r="J2" s="10">
-        <v>0</v>
+        <f>Computation!J2</f>
+        <v>200</v>
       </c>
       <c r="K2" s="10">
-        <v>0</v>
+        <f>Computation!K2</f>
+        <v>200</v>
       </c>
       <c r="L2" s="10">
-        <v>0</v>
+        <f>Computation!L2</f>
+        <v>200</v>
       </c>
       <c r="M2" s="10">
-        <f>'coal retirement'!D42</f>
-        <v>1900</v>
+        <f>Computation!M2</f>
+        <v>200</v>
       </c>
       <c r="N2" s="10">
         <v>0</v>

</xml_diff>